<commit_message>
Saving current state of UI before major overhaul.
</commit_message>
<xml_diff>
--- a/docs/Wiring Table.xlsx
+++ b/docs/Wiring Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\UC Davis\SETI\Thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36511207-4CCA-4880-A602-3D4416043BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4787DC5A-4237-405D-AA2D-3CBCEA0A9D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{764B7A42-86E6-437A-B3DF-A6793BC4B57D}"/>
+    <workbookView xWindow="6465" yWindow="3030" windowWidth="21600" windowHeight="11295" xr2:uid="{764B7A42-86E6-437A-B3DF-A6793BC4B57D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="156">
   <si>
     <t>Signal Name</t>
   </si>
@@ -501,6 +501,9 @@
   </si>
   <si>
     <t>DIO 2-8</t>
+  </si>
+  <si>
+    <t>AMB2</t>
   </si>
 </sst>
 </file>
@@ -1210,7 +1213,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>2</v>
@@ -1454,7 +1457,7 @@
         <v>9</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>66</v>
@@ -1474,7 +1477,7 @@
         <v>9</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>66</v>
@@ -2719,7 +2722,7 @@
         <v>95</v>
       </c>
       <c r="F92" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3849,7 +3852,7 @@
         <v>103</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="E151" s="5" t="s">
         <v>95</v>
@@ -4140,18 +4143,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A143:E143"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A129:E129"/>
     <mergeCell ref="A60:E60"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A143:E143"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A115:E115"/>
-    <mergeCell ref="A81:E81"/>
-    <mergeCell ref="A98:E98"/>
-    <mergeCell ref="A129:E129"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>